<commit_message>
atualizei os dados do 2Q26 da VST
</commit_message>
<xml_diff>
--- a/analise_eua/energia_eletrica/vistra/vst_indicators.xlsx
+++ b/analise_eua/energia_eletrica/vistra/vst_indicators.xlsx
@@ -592,10 +592,10 @@
         <v>2025</v>
       </c>
       <c r="B2" t="n">
-        <v>57.88</v>
+        <v>57.79</v>
       </c>
       <c r="C2" t="n">
-        <v>57.95</v>
+        <v>57.87</v>
       </c>
       <c r="D2" t="n">
         <v>1.73</v>
@@ -607,10 +607,10 @@
         <v>5.32</v>
       </c>
       <c r="G2" t="n">
-        <v>10.72</v>
+        <v>10.7</v>
       </c>
       <c r="H2" t="n">
-        <v>54636428.75000001</v>
+        <v>54558430</v>
       </c>
       <c r="I2" t="n">
         <v>17043</v>
@@ -628,7 +628,7 @@
         <v>3.18</v>
       </c>
       <c r="N2" t="n">
-        <v>14.59</v>
+        <v>14.58</v>
       </c>
       <c r="O2" t="n">
         <v>18.52</v>
@@ -687,13 +687,13 @@
         <v>2024</v>
       </c>
       <c r="B3" t="n">
-        <v>17.76</v>
+        <v>17.73</v>
       </c>
       <c r="C3" t="n">
-        <v>17.76</v>
+        <v>17.74</v>
       </c>
       <c r="D3" t="n">
-        <v>5.63</v>
+        <v>5.64</v>
       </c>
       <c r="E3" t="n">
         <v>6712</v>
@@ -702,10 +702,10 @@
         <v>15.44</v>
       </c>
       <c r="G3" t="n">
-        <v>8.48</v>
+        <v>8.470000000000001</v>
       </c>
       <c r="H3" t="n">
-        <v>47211957.77</v>
+        <v>47146447.86000001</v>
       </c>
       <c r="I3" t="n">
         <v>16298</v>
@@ -723,7 +723,7 @@
         <v>2.71</v>
       </c>
       <c r="N3" t="n">
-        <v>9.279999999999999</v>
+        <v>9.27</v>
       </c>
       <c r="O3" t="n">
         <v>47.74</v>
@@ -782,13 +782,13 @@
         <v>2023</v>
       </c>
       <c r="B4" t="n">
-        <v>9.380000000000001</v>
+        <v>9.369999999999999</v>
       </c>
       <c r="C4" t="n">
-        <v>9.380000000000001</v>
+        <v>9.359999999999999</v>
       </c>
       <c r="D4" t="n">
-        <v>10.67</v>
+        <v>10.68</v>
       </c>
       <c r="E4" t="n">
         <v>4617</v>
@@ -800,7 +800,7 @@
         <v>2.64</v>
       </c>
       <c r="H4" t="n">
-        <v>14006925.48</v>
+        <v>13984739.22</v>
       </c>
       <c r="I4" t="n">
         <v>14402</v>
@@ -818,7 +818,7 @@
         <v>2.05</v>
       </c>
       <c r="N4" t="n">
-        <v>5.39</v>
+        <v>5.38</v>
       </c>
       <c r="O4" t="n">
         <v>28.13</v>
@@ -877,13 +877,13 @@
         <v>2022</v>
       </c>
       <c r="B5" t="n">
-        <v>-7.64</v>
+        <v>-7.63</v>
       </c>
       <c r="C5" t="n">
         <v>0</v>
       </c>
       <c r="D5" t="n">
-        <v>-13.07</v>
+        <v>-13.09</v>
       </c>
       <c r="E5" t="n">
         <v>870</v>
@@ -895,7 +895,7 @@
         <v>1.91</v>
       </c>
       <c r="H5" t="n">
-        <v>9369874.459999999</v>
+        <v>9357201.049999999</v>
       </c>
       <c r="I5" t="n">
         <v>11971</v>
@@ -913,7 +913,7 @@
         <v>2.34</v>
       </c>
       <c r="N5" t="n">
-        <v>23.96</v>
+        <v>23.95</v>
       </c>
       <c r="O5" t="n">
         <v>-25.03</v>
@@ -972,13 +972,13 @@
         <v>2021</v>
       </c>
       <c r="B6" t="n">
-        <v>-7.99</v>
+        <v>-7.98</v>
       </c>
       <c r="C6" t="n">
         <v>0</v>
       </c>
       <c r="D6" t="n">
-        <v>-12.51</v>
+        <v>-12.52</v>
       </c>
       <c r="E6" t="n">
         <v>535</v>
@@ -990,7 +990,7 @@
         <v>1.23</v>
       </c>
       <c r="H6" t="n">
-        <v>10179558.65</v>
+        <v>10165092.2</v>
       </c>
       <c r="I6" t="n">
         <v>10731</v>
@@ -1008,7 +1008,7 @@
         <v>1.13</v>
       </c>
       <c r="N6" t="n">
-        <v>36.57</v>
+        <v>36.54</v>
       </c>
       <c r="O6" t="n">
         <v>-15.37</v>
@@ -1067,13 +1067,13 @@
         <v>2020</v>
       </c>
       <c r="B7" t="n">
-        <v>13.57</v>
+        <v>13.55</v>
       </c>
       <c r="C7" t="n">
-        <v>13.58</v>
+        <v>13.56</v>
       </c>
       <c r="D7" t="n">
-        <v>7.36</v>
+        <v>7.37</v>
       </c>
       <c r="E7" t="n">
         <v>3567</v>
@@ -1085,7 +1085,7 @@
         <v>1.03</v>
       </c>
       <c r="H7" t="n">
-        <v>8629876.880000001</v>
+        <v>8615216.84</v>
       </c>
       <c r="I7" t="n">
         <v>9330</v>
@@ -1103,7 +1103,7 @@
         <v>1.06</v>
       </c>
       <c r="N7" t="n">
-        <v>4.92</v>
+        <v>4.91</v>
       </c>
       <c r="O7" t="n">
         <v>7.6</v>
@@ -1168,7 +1168,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AE14"/>
+  <dimension ref="A1:AE15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1325,1236 +1325,1331 @@
     </row>
     <row r="2">
       <c r="A2" s="2" t="n">
-        <v>46112</v>
+        <v>46203</v>
       </c>
       <c r="B2" t="n">
-        <v>49.35</v>
+        <v>175.19</v>
       </c>
       <c r="C2" t="n">
-        <v>29.25</v>
+        <v>23.19</v>
       </c>
       <c r="D2" t="n">
-        <v>3.42</v>
+        <v>4.31</v>
       </c>
       <c r="E2" t="n">
-        <v>2217</v>
+        <v>1198</v>
       </c>
       <c r="F2" t="n">
-        <v>18.24</v>
+        <v>7.59</v>
       </c>
       <c r="G2" t="n">
-        <v>9.07</v>
+        <v>9.75</v>
       </c>
       <c r="H2" t="n">
-        <v>50785081.92</v>
+        <v>53434039.61</v>
       </c>
       <c r="I2" t="n">
-        <v>19163</v>
+        <v>19595</v>
       </c>
       <c r="J2" t="n">
-        <v>677</v>
+        <v>481</v>
       </c>
       <c r="K2" t="n">
-        <v>18486</v>
+        <v>19114</v>
       </c>
       <c r="L2" t="n">
-        <v>3.15</v>
+        <v>2.98</v>
       </c>
       <c r="M2" t="n">
-        <v>3.3</v>
+        <v>3.49</v>
       </c>
       <c r="N2" t="n">
-        <v>11.79</v>
+        <v>11.3</v>
       </c>
       <c r="O2" t="n">
-        <v>31.09</v>
+        <v>42.19</v>
       </c>
       <c r="P2" t="n">
-        <v>13</v>
+        <v>16.7</v>
       </c>
       <c r="Q2" t="n">
-        <v>1199</v>
+        <v>1023</v>
       </c>
       <c r="R2" t="n">
-        <v>-638</v>
+        <v>-641</v>
       </c>
       <c r="S2" t="n">
-        <v>-706</v>
+        <v>-578</v>
       </c>
       <c r="T2" t="n">
-        <v>322</v>
+        <v>334</v>
       </c>
       <c r="U2" t="n">
-        <v>877</v>
+        <v>689</v>
       </c>
       <c r="V2" t="n">
-        <v>-150</v>
+        <v>-102</v>
       </c>
       <c r="W2" t="n">
         <v>0</v>
       </c>
       <c r="X2" t="n">
-        <v>-150</v>
+        <v>-102</v>
       </c>
       <c r="Y2" t="n">
-        <v>-1043</v>
+        <v>-281</v>
       </c>
       <c r="Z2" t="n">
-        <v>0.62</v>
+        <v>9.31</v>
       </c>
       <c r="AA2" t="n">
-        <v>1715</v>
+        <v>2352</v>
       </c>
       <c r="AB2" t="n">
-        <v>2911</v>
+        <v>3214</v>
       </c>
       <c r="AC2" t="n">
         <v>0.23</v>
       </c>
       <c r="AD2" t="n">
-        <v>7.48</v>
+        <v>25.25</v>
       </c>
       <c r="AE2" t="n">
-        <v>372</v>
+        <v>337</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="n">
-        <v>45930</v>
+        <v>46112</v>
       </c>
       <c r="B3" t="n">
-        <v>101.51</v>
+        <v>49.28</v>
       </c>
       <c r="C3" t="n">
-        <v>25.74</v>
+        <v>29.21</v>
       </c>
       <c r="D3" t="n">
-        <v>3.88</v>
+        <v>3.42</v>
       </c>
       <c r="E3" t="n">
-        <v>1728</v>
+        <v>2217</v>
       </c>
       <c r="F3" t="n">
-        <v>13.12</v>
+        <v>18.24</v>
       </c>
       <c r="G3" t="n">
-        <v>12.7</v>
+        <v>9.06</v>
       </c>
       <c r="H3" t="n">
-        <v>66184779.62</v>
+        <v>50714138.88</v>
       </c>
       <c r="I3" t="n">
-        <v>15988</v>
+        <v>19163</v>
       </c>
       <c r="J3" t="n">
-        <v>638</v>
+        <v>677</v>
       </c>
       <c r="K3" t="n">
-        <v>15350</v>
+        <v>18486</v>
       </c>
       <c r="L3" t="n">
-        <v>2.21</v>
+        <v>3.15</v>
       </c>
       <c r="M3" t="n">
-        <v>2.95</v>
+        <v>3.3</v>
       </c>
       <c r="N3" t="n">
-        <v>11.72</v>
+        <v>11.78</v>
       </c>
       <c r="O3" t="n">
-        <v>49.88</v>
+        <v>31.09</v>
       </c>
       <c r="P3" t="n">
-        <v>22.07</v>
+        <v>13</v>
       </c>
       <c r="Q3" t="n">
-        <v>1467</v>
+        <v>1199</v>
       </c>
       <c r="R3" t="n">
-        <v>-491</v>
+        <v>-638</v>
       </c>
       <c r="S3" t="n">
-        <v>-833</v>
+        <v>-706</v>
       </c>
       <c r="T3" t="n">
-        <v>1009</v>
+        <v>322</v>
       </c>
       <c r="U3" t="n">
-        <v>458</v>
+        <v>877</v>
       </c>
       <c r="V3" t="n">
-        <v>-338</v>
+        <v>-150</v>
       </c>
       <c r="W3" t="n">
         <v>0</v>
       </c>
       <c r="X3" t="n">
-        <v>-338</v>
+        <v>-150</v>
       </c>
       <c r="Y3" t="n">
-        <v>-45</v>
+        <v>-1043</v>
       </c>
       <c r="Z3" t="n">
-        <v>-7.84</v>
+        <v>0.62</v>
       </c>
       <c r="AA3" t="n">
-        <v>1463</v>
+        <v>1715</v>
       </c>
       <c r="AB3" t="n">
-        <v>4387</v>
+        <v>2911</v>
       </c>
       <c r="AC3" t="n">
         <v>0.23</v>
       </c>
       <c r="AD3" t="n">
-        <v>11.81</v>
+        <v>7.48</v>
       </c>
       <c r="AE3" t="n">
-        <v>187</v>
+        <v>372</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="n">
-        <v>45838</v>
+        <v>45930</v>
       </c>
       <c r="B4" t="n">
-        <v>200.39</v>
+        <v>101.37</v>
       </c>
       <c r="C4" t="n">
-        <v>28.73</v>
+        <v>25.71</v>
       </c>
       <c r="D4" t="n">
-        <v>3.48</v>
+        <v>3.89</v>
       </c>
       <c r="E4" t="n">
-        <v>1277</v>
+        <v>1728</v>
       </c>
       <c r="F4" t="n">
-        <v>7.69</v>
+        <v>13.12</v>
       </c>
       <c r="G4" t="n">
-        <v>13.59</v>
+        <v>12.69</v>
       </c>
       <c r="H4" t="n">
-        <v>65528344.14</v>
+        <v>66093317.39000001</v>
       </c>
       <c r="I4" t="n">
-        <v>15770</v>
+        <v>15988</v>
       </c>
       <c r="J4" t="n">
-        <v>495</v>
+        <v>638</v>
       </c>
       <c r="K4" t="n">
-        <v>15275</v>
+        <v>15350</v>
       </c>
       <c r="L4" t="n">
-        <v>2.29</v>
+        <v>2.21</v>
       </c>
       <c r="M4" t="n">
-        <v>3.17</v>
+        <v>2.95</v>
       </c>
       <c r="N4" t="n">
-        <v>12.13</v>
+        <v>11.7</v>
       </c>
       <c r="O4" t="n">
-        <v>47.94</v>
+        <v>49.88</v>
       </c>
       <c r="P4" t="n">
-        <v>21.39</v>
+        <v>22.07</v>
       </c>
       <c r="Q4" t="n">
-        <v>572</v>
+        <v>1467</v>
       </c>
       <c r="R4" t="n">
-        <v>-610</v>
+        <v>-491</v>
       </c>
       <c r="S4" t="n">
-        <v>-63</v>
+        <v>-833</v>
       </c>
       <c r="T4" t="n">
-        <v>-118</v>
+        <v>1009</v>
       </c>
       <c r="U4" t="n">
-        <v>690</v>
+        <v>458</v>
       </c>
       <c r="V4" t="n">
-        <v>-234</v>
+        <v>-338</v>
       </c>
       <c r="W4" t="n">
         <v>0</v>
       </c>
       <c r="X4" t="n">
-        <v>-234</v>
+        <v>-338</v>
       </c>
       <c r="Y4" t="n">
-        <v>-950</v>
+        <v>-45</v>
       </c>
       <c r="Z4" t="n">
-        <v>6.92</v>
+        <v>-7.84</v>
       </c>
       <c r="AA4" t="n">
-        <v>1807</v>
+        <v>1463</v>
       </c>
       <c r="AB4" t="n">
-        <v>3486</v>
+        <v>4387</v>
       </c>
       <c r="AC4" t="n">
-        <v>0.2</v>
+        <v>0.23</v>
       </c>
       <c r="AD4" t="n">
-        <v>21.1</v>
+        <v>11.81</v>
       </c>
       <c r="AE4" t="n">
-        <v>252</v>
+        <v>187</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="n">
-        <v>45747</v>
+        <v>45838</v>
       </c>
       <c r="B5" t="n">
-        <v>-148.14</v>
+        <v>200.11</v>
       </c>
       <c r="C5" t="n">
-        <v>20.64</v>
+        <v>28.69</v>
       </c>
       <c r="D5" t="n">
-        <v>4.84</v>
+        <v>3.49</v>
       </c>
       <c r="E5" t="n">
-        <v>652</v>
+        <v>1277</v>
       </c>
       <c r="F5" t="n">
-        <v>-6.81</v>
+        <v>7.69</v>
       </c>
       <c r="G5" t="n">
-        <v>8.23</v>
+        <v>13.57</v>
       </c>
       <c r="H5" t="n">
-        <v>39702232</v>
+        <v>65436705.6</v>
       </c>
       <c r="I5" t="n">
-        <v>16305</v>
+        <v>15770</v>
       </c>
       <c r="J5" t="n">
-        <v>596</v>
+        <v>495</v>
       </c>
       <c r="K5" t="n">
-        <v>15709</v>
+        <v>15275</v>
       </c>
       <c r="L5" t="n">
-        <v>2.61</v>
+        <v>2.29</v>
       </c>
       <c r="M5" t="n">
-        <v>3.26</v>
+        <v>3.17</v>
       </c>
       <c r="N5" t="n">
-        <v>9.199999999999999</v>
+        <v>12.12</v>
       </c>
       <c r="O5" t="n">
-        <v>40.41</v>
+        <v>47.94</v>
       </c>
       <c r="P5" t="n">
-        <v>18.36</v>
+        <v>21.39</v>
       </c>
       <c r="Q5" t="n">
-        <v>599</v>
+        <v>572</v>
       </c>
       <c r="R5" t="n">
-        <v>-1061</v>
+        <v>-610</v>
       </c>
       <c r="S5" t="n">
-        <v>-164</v>
+        <v>-63</v>
       </c>
       <c r="T5" t="n">
-        <v>-169</v>
+        <v>-118</v>
       </c>
       <c r="U5" t="n">
-        <v>768</v>
+        <v>690</v>
       </c>
       <c r="V5" t="n">
-        <v>2818</v>
+        <v>-234</v>
       </c>
       <c r="W5" t="n">
         <v>0</v>
       </c>
       <c r="X5" t="n">
-        <v>2818</v>
+        <v>-234</v>
       </c>
       <c r="Y5" t="n">
-        <v>-1323</v>
+        <v>-950</v>
       </c>
       <c r="Z5" t="n">
-        <v>85.67</v>
+        <v>6.92</v>
       </c>
       <c r="AA5" t="n">
-        <v>-1449</v>
+        <v>1807</v>
       </c>
       <c r="AB5" t="n">
-        <v>38</v>
+        <v>3486</v>
       </c>
       <c r="AC5" t="n">
-        <v>0.24</v>
+        <v>0.2</v>
       </c>
       <c r="AD5" t="n">
-        <v>-30.97</v>
+        <v>21.1</v>
       </c>
       <c r="AE5" t="n">
-        <v>337</v>
+        <v>252</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="n">
-        <v>45565</v>
+        <v>45747</v>
       </c>
       <c r="B6" t="n">
-        <v>21.35</v>
+        <v>-147.94</v>
       </c>
       <c r="C6" t="n">
-        <v>15.03</v>
+        <v>20.61</v>
       </c>
       <c r="D6" t="n">
-        <v>6.65</v>
+        <v>4.85</v>
       </c>
       <c r="E6" t="n">
-        <v>3302</v>
+        <v>652</v>
       </c>
       <c r="F6" t="n">
-        <v>30.03</v>
+        <v>-6.81</v>
       </c>
       <c r="G6" t="n">
-        <v>7.41</v>
+        <v>8.220000000000001</v>
       </c>
       <c r="H6" t="n">
-        <v>40312693.8</v>
+        <v>39647864</v>
       </c>
       <c r="I6" t="n">
-        <v>14730</v>
+        <v>16305</v>
       </c>
       <c r="J6" t="n">
-        <v>940</v>
+        <v>596</v>
       </c>
       <c r="K6" t="n">
-        <v>13790</v>
+        <v>15709</v>
       </c>
       <c r="L6" t="n">
-        <v>2.06</v>
+        <v>2.61</v>
       </c>
       <c r="M6" t="n">
-        <v>2.53</v>
+        <v>3.26</v>
       </c>
       <c r="N6" t="n">
-        <v>8.07</v>
+        <v>9.19</v>
       </c>
       <c r="O6" t="n">
-        <v>49.99</v>
+        <v>40.41</v>
       </c>
       <c r="P6" t="n">
-        <v>25.68</v>
+        <v>18.36</v>
       </c>
       <c r="Q6" t="n">
-        <v>1702</v>
+        <v>599</v>
       </c>
       <c r="R6" t="n">
-        <v>-762</v>
+        <v>-1061</v>
       </c>
       <c r="S6" t="n">
-        <v>-1661</v>
+        <v>-164</v>
       </c>
       <c r="T6" t="n">
-        <v>1017</v>
+        <v>-169</v>
       </c>
       <c r="U6" t="n">
-        <v>685</v>
+        <v>768</v>
       </c>
       <c r="V6" t="n">
-        <v>2657</v>
+        <v>2818</v>
       </c>
       <c r="W6" t="n">
         <v>0</v>
       </c>
       <c r="X6" t="n">
-        <v>2657</v>
+        <v>2818</v>
       </c>
       <c r="Y6" t="n">
-        <v>871</v>
+        <v>-1323</v>
       </c>
       <c r="Z6" t="n">
-        <v>45.12</v>
+        <v>85.67</v>
       </c>
       <c r="AA6" t="n">
-        <v>2057</v>
+        <v>-1449</v>
       </c>
       <c r="AB6" t="n">
-        <v>1979</v>
+        <v>38</v>
       </c>
       <c r="AC6" t="n">
-        <v>0.23</v>
+        <v>0.24</v>
       </c>
       <c r="AD6" t="n">
-        <v>4.24</v>
+        <v>-30.97</v>
       </c>
       <c r="AE6" t="n">
-        <v>399</v>
+        <v>337</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="n">
-        <v>45473</v>
+        <v>45565</v>
       </c>
       <c r="B7" t="n">
-        <v>80.87</v>
+        <v>21.32</v>
       </c>
       <c r="C7" t="n">
-        <v>23.62</v>
+        <v>15.01</v>
       </c>
       <c r="D7" t="n">
-        <v>4.23</v>
+        <v>6.66</v>
       </c>
       <c r="E7" t="n">
-        <v>1430</v>
+        <v>3302</v>
       </c>
       <c r="F7" t="n">
-        <v>9.49</v>
+        <v>30.03</v>
       </c>
       <c r="G7" t="n">
-        <v>5.28</v>
+        <v>7.4</v>
       </c>
       <c r="H7" t="n">
-        <v>29516262.3</v>
+        <v>40257818.6</v>
       </c>
       <c r="I7" t="n">
-        <v>15886</v>
+        <v>14730</v>
       </c>
       <c r="J7" t="n">
-        <v>1661</v>
+        <v>940</v>
       </c>
       <c r="K7" t="n">
-        <v>14225</v>
+        <v>13790</v>
       </c>
       <c r="L7" t="n">
-        <v>3.19</v>
+        <v>2.06</v>
       </c>
       <c r="M7" t="n">
-        <v>2.54</v>
+        <v>2.53</v>
       </c>
       <c r="N7" t="n">
-        <v>9.81</v>
+        <v>8.06</v>
       </c>
       <c r="O7" t="n">
-        <v>23.39</v>
+        <v>49.99</v>
       </c>
       <c r="P7" t="n">
-        <v>12.8</v>
+        <v>25.68</v>
       </c>
       <c r="Q7" t="n">
-        <v>1196</v>
+        <v>1702</v>
       </c>
       <c r="R7" t="n">
-        <v>-669</v>
+        <v>-762</v>
       </c>
       <c r="S7" t="n">
-        <v>18</v>
+        <v>-1661</v>
       </c>
       <c r="T7" t="n">
-        <v>703</v>
+        <v>1017</v>
       </c>
       <c r="U7" t="n">
-        <v>493</v>
+        <v>685</v>
       </c>
       <c r="V7" t="n">
-        <v>2664</v>
+        <v>2657</v>
       </c>
       <c r="W7" t="n">
         <v>0</v>
       </c>
       <c r="X7" t="n">
-        <v>2664</v>
+        <v>2657</v>
       </c>
       <c r="Y7" t="n">
-        <v>-231</v>
+        <v>871</v>
       </c>
       <c r="Z7" t="n">
-        <v>98.61999999999999</v>
+        <v>45.12</v>
       </c>
       <c r="AA7" t="n">
-        <v>1426</v>
+        <v>2057</v>
       </c>
       <c r="AB7" t="n">
-        <v>-393</v>
+        <v>1979</v>
       </c>
       <c r="AC7" t="n">
-        <v>0.21</v>
+        <v>0.23</v>
       </c>
       <c r="AD7" t="n">
-        <v>20</v>
+        <v>4.24</v>
       </c>
       <c r="AE7" t="n">
-        <v>331</v>
+        <v>399</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="n">
-        <v>45382</v>
+        <v>45473</v>
       </c>
       <c r="B8" t="n">
-        <v>-685.17</v>
+        <v>80.76000000000001</v>
       </c>
       <c r="C8" t="n">
-        <v>15.73</v>
+        <v>23.59</v>
       </c>
       <c r="D8" t="n">
-        <v>6.36</v>
+        <v>4.24</v>
       </c>
       <c r="E8" t="n">
-        <v>641</v>
+        <v>1430</v>
       </c>
       <c r="F8" t="n">
-        <v>-1.15</v>
+        <v>9.49</v>
       </c>
       <c r="G8" t="n">
-        <v>4.24</v>
+        <v>5.27</v>
       </c>
       <c r="H8" t="n">
-        <v>23980943.52</v>
+        <v>29478087.24</v>
       </c>
       <c r="I8" t="n">
-        <v>14747</v>
+        <v>15886</v>
       </c>
       <c r="J8" t="n">
-        <v>1116</v>
+        <v>1661</v>
       </c>
       <c r="K8" t="n">
-        <v>13631</v>
+        <v>14225</v>
       </c>
       <c r="L8" t="n">
-        <v>2.94</v>
+        <v>3.19</v>
       </c>
       <c r="M8" t="n">
-        <v>2.41</v>
+        <v>2.54</v>
       </c>
       <c r="N8" t="n">
-        <v>8.109999999999999</v>
+        <v>9.800000000000001</v>
       </c>
       <c r="O8" t="n">
-        <v>29.03</v>
+        <v>23.39</v>
       </c>
       <c r="P8" t="n">
-        <v>15.15</v>
+        <v>12.8</v>
       </c>
       <c r="Q8" t="n">
-        <v>312</v>
+        <v>1196</v>
       </c>
       <c r="R8" t="n">
-        <v>-3528</v>
+        <v>-669</v>
       </c>
       <c r="S8" t="n">
-        <v>793</v>
+        <v>18</v>
       </c>
       <c r="T8" t="n">
-        <v>-3223</v>
+        <v>703</v>
       </c>
       <c r="U8" t="n">
-        <v>3535</v>
+        <v>493</v>
       </c>
       <c r="V8" t="n">
-        <v>2800</v>
+        <v>2664</v>
       </c>
       <c r="W8" t="n">
         <v>0</v>
       </c>
       <c r="X8" t="n">
-        <v>2800</v>
+        <v>2664</v>
       </c>
       <c r="Y8" t="n">
-        <v>658</v>
+        <v>-231</v>
       </c>
       <c r="Z8" t="n">
-        <v>103.07</v>
+        <v>98.61999999999999</v>
       </c>
       <c r="AA8" t="n">
-        <v>-22</v>
+        <v>1426</v>
       </c>
       <c r="AB8" t="n">
-        <v>-545</v>
+        <v>-393</v>
       </c>
       <c r="AC8" t="n">
-        <v>0.22</v>
+        <v>0.21</v>
       </c>
       <c r="AD8" t="n">
-        <v>-220</v>
+        <v>20</v>
       </c>
       <c r="AE8" t="n">
-        <v>291</v>
+        <v>331</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="n">
-        <v>45199</v>
+        <v>45382</v>
       </c>
       <c r="B9" t="n">
-        <v>23.69</v>
+        <v>-684.27</v>
       </c>
       <c r="C9" t="n">
-        <v>5.34</v>
+        <v>15.7</v>
       </c>
       <c r="D9" t="n">
-        <v>18.74</v>
+        <v>6.37</v>
       </c>
       <c r="E9" t="n">
-        <v>1335</v>
+        <v>641</v>
       </c>
       <c r="F9" t="n">
-        <v>12.29</v>
+        <v>-1.15</v>
       </c>
       <c r="G9" t="n">
-        <v>2.16</v>
+        <v>4.23</v>
       </c>
       <c r="H9" t="n">
-        <v>11891530.8</v>
+        <v>23949536.58</v>
       </c>
       <c r="I9" t="n">
-        <v>13693</v>
+        <v>14747</v>
       </c>
       <c r="J9" t="n">
-        <v>3225</v>
+        <v>1116</v>
       </c>
       <c r="K9" t="n">
-        <v>10468</v>
+        <v>13631</v>
       </c>
       <c r="L9" t="n">
-        <v>1.93</v>
+        <v>2.94</v>
       </c>
       <c r="M9" t="n">
-        <v>1.9</v>
+        <v>2.41</v>
       </c>
       <c r="N9" t="n">
-        <v>4.13</v>
+        <v>8.1</v>
       </c>
       <c r="O9" t="n">
-        <v>42.59</v>
+        <v>29.03</v>
       </c>
       <c r="P9" t="n">
-        <v>21.65</v>
+        <v>15.15</v>
       </c>
       <c r="Q9" t="n">
-        <v>1560</v>
+        <v>312</v>
       </c>
       <c r="R9" t="n">
-        <v>-415</v>
+        <v>-3528</v>
       </c>
       <c r="S9" t="n">
-        <v>1382</v>
+        <v>793</v>
       </c>
       <c r="T9" t="n">
-        <v>1224</v>
+        <v>-3223</v>
       </c>
       <c r="U9" t="n">
-        <v>336</v>
+        <v>3535</v>
       </c>
       <c r="V9" t="n">
-        <v>-405</v>
+        <v>2800</v>
       </c>
       <c r="W9" t="n">
         <v>0</v>
       </c>
       <c r="X9" t="n">
-        <v>-405</v>
+        <v>2800</v>
       </c>
       <c r="Y9" t="n">
-        <v>1951</v>
+        <v>658</v>
       </c>
       <c r="Z9" t="n">
-        <v>-10.11</v>
+        <v>103.07</v>
       </c>
       <c r="AA9" t="n">
-        <v>2535</v>
+        <v>-22</v>
       </c>
       <c r="AB9" t="n">
-        <v>3870</v>
+        <v>-545</v>
       </c>
       <c r="AC9" t="n">
-        <v>0.2</v>
+        <v>0.22</v>
       </c>
       <c r="AD9" t="n">
-        <v>14.94</v>
+        <v>-220</v>
       </c>
       <c r="AE9" t="n">
-        <v>314</v>
+        <v>291</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="n">
-        <v>45107</v>
+        <v>45199</v>
       </c>
       <c r="B10" t="n">
-        <v>19.99</v>
+        <v>23.66</v>
       </c>
       <c r="C10" t="n">
-        <v>16.67</v>
+        <v>5.33</v>
       </c>
       <c r="D10" t="n">
-        <v>6</v>
+        <v>18.77</v>
       </c>
       <c r="E10" t="n">
-        <v>1055</v>
+        <v>1335</v>
       </c>
       <c r="F10" t="n">
-        <v>14.93</v>
+        <v>12.29</v>
       </c>
       <c r="G10" t="n">
-        <v>1.78</v>
+        <v>2.16</v>
       </c>
       <c r="H10" t="n">
-        <v>9514107.560000001</v>
+        <v>11876868</v>
       </c>
       <c r="I10" t="n">
-        <v>11967</v>
+        <v>13693</v>
       </c>
       <c r="J10" t="n">
-        <v>698</v>
+        <v>3225</v>
       </c>
       <c r="K10" t="n">
-        <v>11269</v>
+        <v>10468</v>
       </c>
       <c r="L10" t="n">
-        <v>3.88</v>
+        <v>1.93</v>
       </c>
       <c r="M10" t="n">
-        <v>2.1</v>
+        <v>1.9</v>
       </c>
       <c r="N10" t="n">
-        <v>7.15</v>
+        <v>4.13</v>
       </c>
       <c r="O10" t="n">
-        <v>8.92</v>
+        <v>42.59</v>
       </c>
       <c r="P10" t="n">
-        <v>6.14</v>
+        <v>21.65</v>
       </c>
       <c r="Q10" t="n">
-        <v>1577</v>
+        <v>1560</v>
       </c>
       <c r="R10" t="n">
-        <v>-454</v>
+        <v>-415</v>
       </c>
       <c r="S10" t="n">
-        <v>-998</v>
+        <v>1382</v>
       </c>
       <c r="T10" t="n">
-        <v>1135</v>
+        <v>1224</v>
       </c>
       <c r="U10" t="n">
-        <v>442</v>
+        <v>336</v>
       </c>
       <c r="V10" t="n">
-        <v>-512</v>
+        <v>-405</v>
       </c>
       <c r="W10" t="n">
         <v>0</v>
       </c>
       <c r="X10" t="n">
-        <v>-512</v>
+        <v>-405</v>
       </c>
       <c r="Y10" t="n">
-        <v>1285</v>
+        <v>1951</v>
       </c>
       <c r="Z10" t="n">
-        <v>-108.94</v>
+        <v>-10.11</v>
       </c>
       <c r="AA10" t="n">
-        <v>2370</v>
+        <v>2535</v>
       </c>
       <c r="AB10" t="n">
-        <v>2091</v>
+        <v>3870</v>
       </c>
       <c r="AC10" t="n">
         <v>0.2</v>
       </c>
       <c r="AD10" t="n">
-        <v>15.97</v>
+        <v>14.94</v>
       </c>
       <c r="AE10" t="n">
-        <v>251</v>
+        <v>314</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="n">
-        <v>45016</v>
+        <v>45107</v>
       </c>
       <c r="B11" t="n">
-        <v>12.69</v>
+        <v>19.96</v>
       </c>
       <c r="C11" t="n">
-        <v>0</v>
+        <v>16.65</v>
       </c>
       <c r="D11" t="n">
-        <v>-1.64</v>
+        <v>6.01</v>
       </c>
       <c r="E11" t="n">
-        <v>1608</v>
+        <v>1055</v>
       </c>
       <c r="F11" t="n">
-        <v>15.8</v>
+        <v>14.93</v>
       </c>
       <c r="G11" t="n">
-        <v>1.71</v>
+        <v>1.77</v>
       </c>
       <c r="H11" t="n">
-        <v>8873385.029999999</v>
+        <v>9499189.32</v>
       </c>
       <c r="I11" t="n">
-        <v>11968</v>
+        <v>11967</v>
       </c>
       <c r="J11" t="n">
-        <v>573</v>
+        <v>698</v>
       </c>
       <c r="K11" t="n">
-        <v>11395</v>
+        <v>11269</v>
       </c>
       <c r="L11" t="n">
-        <v>5.41</v>
+        <v>3.88</v>
       </c>
       <c r="M11" t="n">
-        <v>2.19</v>
+        <v>2.1</v>
       </c>
       <c r="N11" t="n">
-        <v>9.619999999999999</v>
+        <v>7.14</v>
       </c>
       <c r="O11" t="n">
-        <v>-5.44</v>
+        <v>8.92</v>
       </c>
       <c r="P11" t="n">
-        <v>-0.17</v>
+        <v>6.14</v>
       </c>
       <c r="Q11" t="n">
-        <v>1435</v>
+        <v>1577</v>
       </c>
       <c r="R11" t="n">
-        <v>-513</v>
+        <v>-454</v>
       </c>
       <c r="S11" t="n">
-        <v>-874</v>
+        <v>-998</v>
       </c>
       <c r="T11" t="n">
-        <v>951</v>
+        <v>1135</v>
       </c>
       <c r="U11" t="n">
-        <v>484</v>
+        <v>442</v>
       </c>
       <c r="V11" t="n">
-        <v>-659</v>
+        <v>-512</v>
       </c>
       <c r="W11" t="n">
         <v>0</v>
       </c>
       <c r="X11" t="n">
-        <v>-659</v>
+        <v>-512</v>
       </c>
       <c r="Y11" t="n">
-        <v>1350</v>
+        <v>1285</v>
       </c>
       <c r="Z11" t="n">
-        <v>5313.33</v>
+        <v>-108.94</v>
       </c>
       <c r="AA11" t="n">
-        <v>1920</v>
+        <v>2370</v>
       </c>
       <c r="AB11" t="n">
-        <v>1648</v>
+        <v>2091</v>
       </c>
       <c r="AC11" t="n">
         <v>0.2</v>
       </c>
       <c r="AD11" t="n">
-        <v>11.02</v>
+        <v>15.97</v>
       </c>
       <c r="AE11" t="n">
-        <v>301</v>
+        <v>251</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="n">
-        <v>44834</v>
+        <v>45016</v>
       </c>
       <c r="B12" t="n">
-        <v>12.34</v>
+        <v>12.68</v>
       </c>
       <c r="C12" t="n">
         <v>0</v>
       </c>
       <c r="D12" t="n">
-        <v>-10.99</v>
+        <v>-1.65</v>
       </c>
       <c r="E12" t="n">
-        <v>1415</v>
+        <v>1608</v>
       </c>
       <c r="F12" t="n">
-        <v>12.98</v>
+        <v>15.8</v>
       </c>
       <c r="G12" t="n">
-        <v>1.48</v>
+        <v>1.7</v>
       </c>
       <c r="H12" t="n">
-        <v>8242158.960000001</v>
+        <v>8861876.1</v>
       </c>
       <c r="I12" t="n">
-        <v>11985</v>
+        <v>11968</v>
       </c>
       <c r="J12" t="n">
-        <v>568</v>
+        <v>573</v>
       </c>
       <c r="K12" t="n">
-        <v>11417</v>
+        <v>11395</v>
       </c>
       <c r="L12" t="n">
-        <v>9.52</v>
+        <v>5.41</v>
       </c>
       <c r="M12" t="n">
-        <v>2.05</v>
+        <v>2.19</v>
       </c>
       <c r="N12" t="n">
-        <v>16.4</v>
+        <v>9.619999999999999</v>
       </c>
       <c r="O12" t="n">
-        <v>-17.47</v>
+        <v>-5.44</v>
       </c>
       <c r="P12" t="n">
-        <v>-6.77</v>
+        <v>-0.17</v>
       </c>
       <c r="Q12" t="n">
-        <v>815</v>
+        <v>1435</v>
       </c>
       <c r="R12" t="n">
-        <v>-277</v>
+        <v>-513</v>
       </c>
       <c r="S12" t="n">
-        <v>-1877</v>
+        <v>-874</v>
       </c>
       <c r="T12" t="n">
-        <v>519</v>
+        <v>951</v>
       </c>
       <c r="U12" t="n">
-        <v>296</v>
+        <v>484</v>
       </c>
       <c r="V12" t="n">
-        <v>-1004</v>
+        <v>-659</v>
       </c>
       <c r="W12" t="n">
         <v>0</v>
       </c>
       <c r="X12" t="n">
-        <v>-1004</v>
+        <v>-659</v>
       </c>
       <c r="Y12" t="n">
-        <v>1234</v>
+        <v>1350</v>
       </c>
       <c r="Z12" t="n">
-        <v>68.88</v>
+        <v>5313.33</v>
       </c>
       <c r="AA12" t="n">
-        <v>-273</v>
+        <v>1920</v>
       </c>
       <c r="AB12" t="n">
-        <v>-386</v>
+        <v>1648</v>
       </c>
       <c r="AC12" t="n">
-        <v>0.18</v>
+        <v>0.2</v>
       </c>
       <c r="AD12" t="n">
-        <v>11.23</v>
+        <v>11.02</v>
       </c>
       <c r="AE12" t="n">
-        <v>396</v>
+        <v>301</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="n">
-        <v>44742</v>
+        <v>44834</v>
       </c>
       <c r="B13" t="n">
-        <v>-6.77</v>
+        <v>12.32</v>
       </c>
       <c r="C13" t="n">
         <v>0</v>
       </c>
       <c r="D13" t="n">
-        <v>-17.33</v>
+        <v>-11.01</v>
       </c>
       <c r="E13" t="n">
-        <v>-1171</v>
+        <v>1415</v>
       </c>
       <c r="F13" t="n">
-        <v>-85.95999999999999</v>
+        <v>12.98</v>
       </c>
       <c r="G13" t="n">
-        <v>1.71</v>
+        <v>1.47</v>
       </c>
       <c r="H13" t="n">
-        <v>9236233.359999999</v>
+        <v>8229746.07</v>
       </c>
       <c r="I13" t="n">
-        <v>11990</v>
+        <v>11985</v>
       </c>
       <c r="J13" t="n">
-        <v>1907</v>
+        <v>568</v>
       </c>
       <c r="K13" t="n">
-        <v>10083</v>
+        <v>11417</v>
       </c>
       <c r="L13" t="n">
-        <v>33.17</v>
+        <v>9.52</v>
       </c>
       <c r="M13" t="n">
-        <v>1.87</v>
+        <v>2.05</v>
       </c>
       <c r="N13" t="n">
-        <v>63.55</v>
+        <v>16.39</v>
       </c>
       <c r="O13" t="n">
-        <v>-29.8</v>
+        <v>-17.47</v>
       </c>
       <c r="P13" t="n">
-        <v>-13.65</v>
+        <v>-6.77</v>
       </c>
       <c r="Q13" t="n">
-        <v>-1314</v>
+        <v>815</v>
       </c>
       <c r="R13" t="n">
-        <v>-129</v>
+        <v>-277</v>
       </c>
       <c r="S13" t="n">
-        <v>2293</v>
+        <v>-1877</v>
       </c>
       <c r="T13" t="n">
-        <v>-1554</v>
+        <v>519</v>
       </c>
       <c r="U13" t="n">
-        <v>240</v>
+        <v>296</v>
       </c>
       <c r="V13" t="n">
-        <v>-883</v>
+        <v>-1004</v>
       </c>
       <c r="W13" t="n">
         <v>0</v>
       </c>
       <c r="X13" t="n">
-        <v>-883</v>
+        <v>-1004</v>
       </c>
       <c r="Y13" t="n">
-        <v>654</v>
+        <v>1234</v>
       </c>
       <c r="Z13" t="n">
-        <v>-50.89</v>
+        <v>68.88</v>
       </c>
       <c r="AA13" t="n">
-        <v>-1737</v>
+        <v>-273</v>
       </c>
       <c r="AB13" t="n">
-        <v>-3410</v>
+        <v>-386</v>
       </c>
       <c r="AC13" t="n">
-        <v>0.17</v>
+        <v>0.18</v>
       </c>
       <c r="AD13" t="n">
-        <v>-5.49</v>
+        <v>11.23</v>
       </c>
       <c r="AE13" t="n">
-        <v>484</v>
+        <v>396</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="n">
-        <v>44651</v>
+        <v>44742</v>
       </c>
       <c r="B14" t="n">
-        <v>-34.42</v>
+        <v>-6.76</v>
       </c>
       <c r="C14" t="n">
         <v>0</v>
       </c>
       <c r="D14" t="n">
-        <v>-21.92</v>
+        <v>-17.36</v>
       </c>
       <c r="E14" t="n">
-        <v>254</v>
+        <v>-1171</v>
       </c>
       <c r="F14" t="n">
-        <v>-9.119999999999999</v>
+        <v>-85.95999999999999</v>
       </c>
       <c r="G14" t="n">
-        <v>1.34</v>
+        <v>1.71</v>
       </c>
       <c r="H14" t="n">
-        <v>9808817.16</v>
+        <v>9223357.569999998</v>
       </c>
       <c r="I14" t="n">
-        <v>10597</v>
+        <v>11990</v>
       </c>
       <c r="J14" t="n">
-        <v>1057</v>
+        <v>1907</v>
       </c>
       <c r="K14" t="n">
-        <v>9540</v>
+        <v>10083</v>
       </c>
       <c r="L14" t="n">
-        <v>-15.98</v>
+        <v>33.17</v>
       </c>
       <c r="M14" t="n">
-        <v>1.31</v>
+        <v>1.87</v>
       </c>
       <c r="N14" t="n">
-        <v>-32.41</v>
+        <v>63.51</v>
       </c>
       <c r="O14" t="n">
-        <v>-31.3</v>
+        <v>-29.8</v>
       </c>
       <c r="P14" t="n">
-        <v>-18.72</v>
+        <v>-13.65</v>
       </c>
       <c r="Q14" t="n">
-        <v>591</v>
+        <v>-1314</v>
       </c>
       <c r="R14" t="n">
-        <v>-480</v>
+        <v>-129</v>
       </c>
       <c r="S14" t="n">
-        <v>-413</v>
+        <v>2293</v>
       </c>
       <c r="T14" t="n">
-        <v>218</v>
+        <v>-1554</v>
       </c>
       <c r="U14" t="n">
-        <v>373</v>
+        <v>240</v>
       </c>
       <c r="V14" t="n">
-        <v>-930</v>
+        <v>-883</v>
       </c>
       <c r="W14" t="n">
         <v>0</v>
       </c>
       <c r="X14" t="n">
-        <v>-930</v>
+        <v>-883</v>
       </c>
       <c r="Y14" t="n">
-        <v>1048</v>
+        <v>654</v>
       </c>
       <c r="Z14" t="n">
-        <v>29.16</v>
+        <v>-50.89</v>
       </c>
       <c r="AA14" t="n">
-        <v>-1674</v>
+        <v>-1737</v>
       </c>
       <c r="AB14" t="n">
-        <v>-2366</v>
+        <v>-3410</v>
       </c>
       <c r="AC14" t="n">
         <v>0.17</v>
       </c>
       <c r="AD14" t="n">
+        <v>-5.49</v>
+      </c>
+      <c r="AE14" t="n">
+        <v>484</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="n">
+        <v>44651</v>
+      </c>
+      <c r="B15" t="n">
+        <v>-34.37</v>
+      </c>
+      <c r="C15" t="n">
+        <v>0</v>
+      </c>
+      <c r="D15" t="n">
+        <v>-21.95</v>
+      </c>
+      <c r="E15" t="n">
+        <v>254</v>
+      </c>
+      <c r="F15" t="n">
+        <v>-9.119999999999999</v>
+      </c>
+      <c r="G15" t="n">
+        <v>1.34</v>
+      </c>
+      <c r="H15" t="n">
+        <v>9795269.07</v>
+      </c>
+      <c r="I15" t="n">
+        <v>10597</v>
+      </c>
+      <c r="J15" t="n">
+        <v>1057</v>
+      </c>
+      <c r="K15" t="n">
+        <v>9540</v>
+      </c>
+      <c r="L15" t="n">
+        <v>-15.98</v>
+      </c>
+      <c r="M15" t="n">
+        <v>1.31</v>
+      </c>
+      <c r="N15" t="n">
+        <v>-32.39</v>
+      </c>
+      <c r="O15" t="n">
+        <v>-31.3</v>
+      </c>
+      <c r="P15" t="n">
+        <v>-18.72</v>
+      </c>
+      <c r="Q15" t="n">
+        <v>591</v>
+      </c>
+      <c r="R15" t="n">
+        <v>-480</v>
+      </c>
+      <c r="S15" t="n">
+        <v>-413</v>
+      </c>
+      <c r="T15" t="n">
+        <v>218</v>
+      </c>
+      <c r="U15" t="n">
+        <v>373</v>
+      </c>
+      <c r="V15" t="n">
+        <v>-930</v>
+      </c>
+      <c r="W15" t="n">
+        <v>0</v>
+      </c>
+      <c r="X15" t="n">
+        <v>-930</v>
+      </c>
+      <c r="Y15" t="n">
+        <v>1048</v>
+      </c>
+      <c r="Z15" t="n">
+        <v>29.16</v>
+      </c>
+      <c r="AA15" t="n">
+        <v>-1674</v>
+      </c>
+      <c r="AB15" t="n">
+        <v>-2366</v>
+      </c>
+      <c r="AC15" t="n">
+        <v>0.17</v>
+      </c>
+      <c r="AD15" t="n">
         <v>-27.02</v>
       </c>
-      <c r="AE14" t="n">
+      <c r="AE15" t="n">
         <v>710</v>
       </c>
     </row>

</xml_diff>